<commit_message>
Actualización de las demás gráficas
</commit_message>
<xml_diff>
--- a/jjjjj.xlsx
+++ b/jjjjj.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Laura\Documents\GitHub\Costo mano de obra\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://molt246-my.sharepoint.com/personal/lauras_molt_com_co/Documents/Documentos/GitHub/Costo mano de obra/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C230622A-3048-427C-9ED0-335E7E02A5BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{C230622A-3048-427C-9ED0-335E7E02A5BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF90B21D-6C7B-4059-BB98-8EB927EF4CB1}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6420" yWindow="576" windowWidth="15108" windowHeight="10908" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -7447,7 +7447,7 @@
         <cdr:cNvPr id="2" name="Rectángulo 1">
           <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FBB5F673-1D67-F752-A08A-5FA534D32DF4}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{07A16E30-00E0-B2D8-9CCF-AB3FF217BA52}"/>
             </a:ext>
           </a:extLst>
         </cdr:cNvPr>
@@ -8964,7 +8964,13 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{393F98C7-64BD-42A7-8F61-B63601B7BCE0}" name="Tabla1" displayName="Tabla1" ref="A1:W497" totalsRowCount="1">
-  <autoFilter ref="A1:W496" xr:uid="{393F98C7-64BD-42A7-8F61-B63601B7BCE0}"/>
+  <autoFilter ref="A1:W496" xr:uid="{393F98C7-64BD-42A7-8F61-B63601B7BCE0}">
+    <filterColumn colId="6">
+      <filters>
+        <filter val="Medias Cuarto Frio"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:W496">
     <sortCondition descending="1" ref="V1:V496"/>
   </sortState>
@@ -9390,7 +9396,7 @@
         <v>1373</v>
       </c>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>6492</v>
       </c>
@@ -9466,7 +9472,7 @@
         <v>1800000</v>
       </c>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>6492</v>
       </c>
@@ -9542,7 +9548,7 @@
         <v>1800000</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>6492</v>
       </c>
@@ -9618,7 +9624,7 @@
         <v>1600000</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>6492</v>
       </c>
@@ -9694,7 +9700,7 @@
         <v>1600000</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>6533</v>
       </c>
@@ -9770,7 +9776,7 @@
         <v>1200000</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6485</v>
       </c>
@@ -9846,7 +9852,7 @@
         <v>1200000</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>6485</v>
       </c>
@@ -9922,7 +9928,7 @@
         <v>1200000</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>6533</v>
       </c>
@@ -9998,7 +10004,7 @@
         <v>1200000</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>6533</v>
       </c>
@@ -10074,7 +10080,7 @@
         <v>800000</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>6533</v>
       </c>
@@ -10150,7 +10156,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>6533</v>
       </c>
@@ -10226,7 +10232,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>6425</v>
       </c>
@@ -10302,7 +10308,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>6430</v>
       </c>
@@ -10378,7 +10384,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>6430</v>
       </c>
@@ -10454,7 +10460,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>6430</v>
       </c>
@@ -10530,7 +10536,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>6492</v>
       </c>
@@ -10606,7 +10612,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>6492</v>
       </c>
@@ -10682,7 +10688,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>6492</v>
       </c>
@@ -10758,7 +10764,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>6492</v>
       </c>
@@ -10834,7 +10840,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>6533</v>
       </c>
@@ -10910,7 +10916,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>6492</v>
       </c>
@@ -10986,7 +10992,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>6492</v>
       </c>
@@ -11062,7 +11068,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>6492</v>
       </c>
@@ -11138,7 +11144,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>6492</v>
       </c>
@@ -11214,7 +11220,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>6492</v>
       </c>
@@ -11290,7 +11296,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>6492</v>
       </c>
@@ -11366,7 +11372,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>6297</v>
       </c>
@@ -11518,7 +11524,7 @@
         <v>200000</v>
       </c>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>6620</v>
       </c>
@@ -11594,7 +11600,7 @@
         <v>200000</v>
       </c>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>6487</v>
       </c>
@@ -11670,7 +11676,7 @@
         <v>200000</v>
       </c>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>6425</v>
       </c>
@@ -11746,7 +11752,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>6543</v>
       </c>
@@ -11822,7 +11828,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>6487</v>
       </c>
@@ -11898,7 +11904,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>6541</v>
       </c>
@@ -11974,7 +11980,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>6373</v>
       </c>
@@ -12050,7 +12056,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>6492</v>
       </c>
@@ -12126,7 +12132,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>6492</v>
       </c>
@@ -12202,7 +12208,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>6485</v>
       </c>
@@ -12278,7 +12284,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>6485</v>
       </c>
@@ -12354,7 +12360,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>6383</v>
       </c>
@@ -12430,7 +12436,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>6371</v>
       </c>
@@ -12506,7 +12512,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>6541</v>
       </c>
@@ -12582,7 +12588,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>6370</v>
       </c>
@@ -12658,7 +12664,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>6491</v>
       </c>
@@ -12734,7 +12740,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>6543</v>
       </c>
@@ -12810,7 +12816,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>6496</v>
       </c>
@@ -12886,7 +12892,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>6496</v>
       </c>
@@ -12962,7 +12968,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>6496</v>
       </c>
@@ -13038,7 +13044,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>6492</v>
       </c>
@@ -13114,7 +13120,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>6492</v>
       </c>
@@ -13190,7 +13196,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>6486</v>
       </c>
@@ -13266,7 +13272,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>6428</v>
       </c>
@@ -13342,7 +13348,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>6374</v>
       </c>
@@ -13418,7 +13424,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>6484</v>
       </c>
@@ -13494,7 +13500,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>6492</v>
       </c>
@@ -13570,7 +13576,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>6492</v>
       </c>
@@ -13646,7 +13652,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>6492</v>
       </c>
@@ -13722,7 +13728,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>6492</v>
       </c>
@@ -13798,7 +13804,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>6492</v>
       </c>
@@ -13874,7 +13880,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>6492</v>
       </c>
@@ -13950,7 +13956,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>6371</v>
       </c>
@@ -14026,7 +14032,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>6541</v>
       </c>
@@ -14102,7 +14108,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>6618</v>
       </c>
@@ -14178,7 +14184,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>6618</v>
       </c>
@@ -14254,7 +14260,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>6487</v>
       </c>
@@ -14330,7 +14336,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>6378</v>
       </c>
@@ -14406,7 +14412,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>6378</v>
       </c>
@@ -14482,7 +14488,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>6492</v>
       </c>
@@ -14558,7 +14564,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>6492</v>
       </c>
@@ -14634,7 +14640,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>6379</v>
       </c>
@@ -14710,7 +14716,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>6492</v>
       </c>
@@ -14786,7 +14792,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>6492</v>
       </c>
@@ -14862,7 +14868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>6371</v>
       </c>
@@ -14938,7 +14944,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>6487</v>
       </c>
@@ -15014,7 +15020,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>6611</v>
       </c>
@@ -15090,7 +15096,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>6433</v>
       </c>
@@ -15166,7 +15172,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>6421</v>
       </c>
@@ -15242,7 +15248,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>6486</v>
       </c>
@@ -15318,7 +15324,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>6379</v>
       </c>
@@ -15394,7 +15400,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>6484</v>
       </c>
@@ -15470,7 +15476,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>6492</v>
       </c>
@@ -15546,7 +15552,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>6492</v>
       </c>
@@ -15622,7 +15628,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>6492</v>
       </c>
@@ -15698,7 +15704,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>6492</v>
       </c>
@@ -15774,7 +15780,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>6297</v>
       </c>
@@ -15850,7 +15856,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>6415</v>
       </c>
@@ -15926,7 +15932,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>6492</v>
       </c>
@@ -16002,7 +16008,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>6492</v>
       </c>
@@ -16078,7 +16084,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>6486</v>
       </c>
@@ -16154,7 +16160,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>6364</v>
       </c>
@@ -16230,7 +16236,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>6439</v>
       </c>
@@ -16306,7 +16312,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>6492</v>
       </c>
@@ -16382,7 +16388,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>6492</v>
       </c>
@@ -16534,7 +16540,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>6486</v>
       </c>
@@ -16610,7 +16616,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>6486</v>
       </c>
@@ -16686,7 +16692,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>6524</v>
       </c>
@@ -16762,7 +16768,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>6433</v>
       </c>
@@ -16838,7 +16844,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100">
         <v>6492</v>
       </c>
@@ -16914,7 +16920,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101">
         <v>6492</v>
       </c>
@@ -16990,7 +16996,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102">
         <v>6492</v>
       </c>
@@ -17066,7 +17072,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103">
         <v>6492</v>
       </c>
@@ -17142,7 +17148,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104">
         <v>6487</v>
       </c>
@@ -17218,7 +17224,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105">
         <v>6486</v>
       </c>
@@ -17294,7 +17300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A106">
         <v>6485</v>
       </c>
@@ -17370,7 +17376,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107">
         <v>6485</v>
       </c>
@@ -17446,7 +17452,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108">
         <v>6486</v>
       </c>
@@ -17522,7 +17528,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109">
         <v>6379</v>
       </c>
@@ -17598,7 +17604,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110">
         <v>6371</v>
       </c>
@@ -17674,7 +17680,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111">
         <v>6484</v>
       </c>
@@ -17750,7 +17756,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A112">
         <v>6611</v>
       </c>
@@ -17826,7 +17832,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113">
         <v>6487</v>
       </c>
@@ -17902,7 +17908,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A114">
         <v>6492</v>
       </c>
@@ -17978,7 +17984,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A115">
         <v>6492</v>
       </c>
@@ -18054,7 +18060,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A116">
         <v>6526</v>
       </c>
@@ -18130,7 +18136,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A117">
         <v>6487</v>
       </c>
@@ -18206,7 +18212,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A118">
         <v>6486</v>
       </c>
@@ -18282,7 +18288,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119">
         <v>6487</v>
       </c>
@@ -18358,7 +18364,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120">
         <v>6421</v>
       </c>
@@ -18434,7 +18440,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A121">
         <v>6378</v>
       </c>
@@ -18510,7 +18516,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A122">
         <v>6378</v>
       </c>
@@ -18586,7 +18592,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123">
         <v>6492</v>
       </c>
@@ -18662,7 +18668,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A124">
         <v>6492</v>
       </c>
@@ -18738,7 +18744,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A125">
         <v>6486</v>
       </c>
@@ -18814,7 +18820,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A126">
         <v>6379</v>
       </c>
@@ -18890,7 +18896,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A127">
         <v>6528</v>
       </c>
@@ -18966,7 +18972,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A128">
         <v>6297</v>
       </c>
@@ -19042,7 +19048,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A129">
         <v>6421</v>
       </c>
@@ -19118,7 +19124,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A130">
         <v>6421</v>
       </c>
@@ -19194,7 +19200,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A131">
         <v>6439</v>
       </c>
@@ -19270,7 +19276,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A132">
         <v>6439</v>
       </c>
@@ -19346,7 +19352,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A133">
         <v>6439</v>
       </c>
@@ -19422,7 +19428,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A134">
         <v>6618</v>
       </c>
@@ -19498,7 +19504,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A135">
         <v>6618</v>
       </c>
@@ -19574,7 +19580,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A136">
         <v>6381</v>
       </c>
@@ -19650,7 +19656,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A137">
         <v>6524</v>
       </c>
@@ -19726,7 +19732,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A138">
         <v>6524</v>
       </c>
@@ -19802,7 +19808,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A139">
         <v>6492</v>
       </c>
@@ -19878,7 +19884,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A140">
         <v>6492</v>
       </c>
@@ -19954,7 +19960,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A141">
         <v>6439</v>
       </c>
@@ -20030,7 +20036,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A142">
         <v>6439</v>
       </c>
@@ -20106,7 +20112,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A143">
         <v>6492</v>
       </c>
@@ -20182,7 +20188,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A144">
         <v>6492</v>
       </c>
@@ -20258,7 +20264,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A145">
         <v>6383</v>
       </c>
@@ -20334,7 +20340,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A146">
         <v>6382</v>
       </c>
@@ -20410,7 +20416,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A147">
         <v>6382</v>
       </c>
@@ -20486,7 +20492,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A148">
         <v>6382</v>
       </c>
@@ -20562,7 +20568,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A149">
         <v>6486</v>
       </c>
@@ -20638,7 +20644,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A150">
         <v>6433</v>
       </c>
@@ -20714,7 +20720,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A151">
         <v>6433</v>
       </c>
@@ -20790,7 +20796,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A152">
         <v>6433</v>
       </c>
@@ -20866,7 +20872,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A153">
         <v>6492</v>
       </c>
@@ -20942,7 +20948,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A154">
         <v>6492</v>
       </c>
@@ -21018,7 +21024,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A155">
         <v>6492</v>
       </c>
@@ -21094,7 +21100,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A156">
         <v>6492</v>
       </c>
@@ -21170,7 +21176,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A157">
         <v>6533</v>
       </c>
@@ -21246,7 +21252,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A158">
         <v>6524</v>
       </c>
@@ -21398,7 +21404,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A160">
         <v>6421</v>
       </c>
@@ -21474,7 +21480,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A161">
         <v>6618</v>
       </c>
@@ -21550,7 +21556,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A162">
         <v>6517</v>
       </c>
@@ -21626,7 +21632,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A163">
         <v>6523</v>
       </c>
@@ -21702,7 +21708,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A164">
         <v>6523</v>
       </c>
@@ -21778,7 +21784,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A165">
         <v>6523</v>
       </c>
@@ -21854,7 +21860,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A166">
         <v>6523</v>
       </c>
@@ -21930,7 +21936,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A167">
         <v>6433</v>
       </c>
@@ -22006,7 +22012,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A168">
         <v>6379</v>
       </c>
@@ -22082,7 +22088,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A169">
         <v>6540</v>
       </c>
@@ -22158,7 +22164,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A170">
         <v>6540</v>
       </c>
@@ -22234,7 +22240,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A171">
         <v>6540</v>
       </c>
@@ -22310,7 +22316,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A172">
         <v>6421</v>
       </c>
@@ -22386,7 +22392,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A173">
         <v>6384</v>
       </c>
@@ -22462,7 +22468,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A174">
         <v>6382</v>
       </c>
@@ -22538,7 +22544,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A175">
         <v>6538</v>
       </c>
@@ -22614,7 +22620,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A176">
         <v>6538</v>
       </c>
@@ -22690,7 +22696,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A177">
         <v>6492</v>
       </c>
@@ -22766,7 +22772,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A178">
         <v>6492</v>
       </c>
@@ -22842,7 +22848,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A179">
         <v>6379</v>
       </c>
@@ -22918,7 +22924,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A180">
         <v>6379</v>
       </c>
@@ -22994,7 +23000,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A181">
         <v>6384</v>
       </c>
@@ -23070,7 +23076,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A182">
         <v>6421</v>
       </c>
@@ -23146,7 +23152,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A183">
         <v>6421</v>
       </c>
@@ -23222,7 +23228,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A184">
         <v>6376</v>
       </c>
@@ -23298,7 +23304,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A185">
         <v>6376</v>
       </c>
@@ -23374,7 +23380,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A186">
         <v>6376</v>
       </c>
@@ -23450,7 +23456,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A187">
         <v>6382</v>
       </c>
@@ -23526,7 +23532,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A188">
         <v>6382</v>
       </c>
@@ -23602,7 +23608,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A189">
         <v>6363</v>
       </c>
@@ -23678,7 +23684,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A190">
         <v>6363</v>
       </c>
@@ -23754,7 +23760,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A191">
         <v>6384</v>
       </c>
@@ -23830,7 +23836,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A192">
         <v>6540</v>
       </c>
@@ -23906,7 +23912,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A193">
         <v>6540</v>
       </c>
@@ -23982,7 +23988,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A194">
         <v>6540</v>
       </c>
@@ -24058,7 +24064,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A195">
         <v>6439</v>
       </c>
@@ -24134,7 +24140,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A196">
         <v>6439</v>
       </c>
@@ -24210,7 +24216,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A197">
         <v>6382</v>
       </c>
@@ -24286,7 +24292,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A198">
         <v>6382</v>
       </c>
@@ -24362,7 +24368,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A199">
         <v>6379</v>
       </c>
@@ -24438,7 +24444,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A200">
         <v>6493</v>
       </c>
@@ -24514,7 +24520,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A201">
         <v>6493</v>
       </c>
@@ -24590,7 +24596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A202">
         <v>6379</v>
       </c>
@@ -24666,7 +24672,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A203">
         <v>6384</v>
       </c>
@@ -24742,7 +24748,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A204">
         <v>6379</v>
       </c>
@@ -24818,7 +24824,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="205" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A205">
         <v>6492</v>
       </c>
@@ -24894,7 +24900,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="206" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A206">
         <v>6492</v>
       </c>
@@ -24970,7 +24976,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="207" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A207">
         <v>6616</v>
       </c>
@@ -25046,7 +25052,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="208" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A208">
         <v>6616</v>
       </c>
@@ -25122,7 +25128,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="209" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A209">
         <v>6383</v>
       </c>
@@ -25198,7 +25204,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="210" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A210">
         <v>6489</v>
       </c>
@@ -25274,7 +25280,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="211" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A211">
         <v>6489</v>
       </c>
@@ -25350,7 +25356,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="212" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A212">
         <v>6616</v>
       </c>
@@ -25426,7 +25432,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A213">
         <v>6383</v>
       </c>
@@ -25502,7 +25508,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="214" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A214">
         <v>6383</v>
       </c>
@@ -25578,7 +25584,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="215" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A215">
         <v>6485</v>
       </c>
@@ -25654,7 +25660,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="216" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A216">
         <v>6485</v>
       </c>
@@ -25730,7 +25736,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="217" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A217">
         <v>6485</v>
       </c>
@@ -25806,7 +25812,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="218" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A218">
         <v>6485</v>
       </c>
@@ -25882,7 +25888,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="219" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A219">
         <v>6528</v>
       </c>
@@ -25958,7 +25964,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="220" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A220">
         <v>6487</v>
       </c>
@@ -26034,7 +26040,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="221" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A221">
         <v>6383</v>
       </c>
@@ -26110,7 +26116,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="222" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A222">
         <v>6487</v>
       </c>
@@ -26186,7 +26192,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="223" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A223">
         <v>6485</v>
       </c>
@@ -26262,7 +26268,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="224" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A224">
         <v>6485</v>
       </c>
@@ -26338,7 +26344,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="225" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A225">
         <v>6421</v>
       </c>
@@ -26414,7 +26420,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="226" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A226">
         <v>6435</v>
       </c>
@@ -26490,7 +26496,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="227" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A227">
         <v>6381</v>
       </c>
@@ -26566,7 +26572,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="228" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A228">
         <v>6484</v>
       </c>
@@ -26642,7 +26648,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="229" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A229">
         <v>6486</v>
       </c>
@@ -26718,7 +26724,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="230" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A230">
         <v>6433</v>
       </c>
@@ -26794,7 +26800,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="231" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A231">
         <v>6485</v>
       </c>
@@ -26870,7 +26876,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="232" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A232">
         <v>6485</v>
       </c>
@@ -26946,7 +26952,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="233" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A233">
         <v>6485</v>
       </c>
@@ -27022,7 +27028,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="234" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A234">
         <v>6485</v>
       </c>
@@ -27098,7 +27104,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="235" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A235">
         <v>6436</v>
       </c>
@@ -27174,7 +27180,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="236" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A236">
         <v>6383</v>
       </c>
@@ -27250,7 +27256,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="237" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A237">
         <v>6379</v>
       </c>
@@ -27326,7 +27332,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="238" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A238">
         <v>6383</v>
       </c>
@@ -27402,7 +27408,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="239" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A239">
         <v>6383</v>
       </c>
@@ -27478,7 +27484,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="240" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A240">
         <v>6485</v>
       </c>
@@ -27554,7 +27560,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="241" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A241">
         <v>6485</v>
       </c>
@@ -27630,7 +27636,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="242" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A242">
         <v>6484</v>
       </c>
@@ -27706,7 +27712,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="243" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A243">
         <v>6526</v>
       </c>
@@ -27782,7 +27788,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="244" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A244">
         <v>6487</v>
       </c>
@@ -27858,7 +27864,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="245" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A245">
         <v>6436</v>
       </c>
@@ -27934,7 +27940,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="246" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A246">
         <v>6524</v>
       </c>
@@ -28010,7 +28016,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="247" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A247">
         <v>6503</v>
       </c>
@@ -28086,7 +28092,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="248" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A248">
         <v>6503</v>
       </c>
@@ -28162,7 +28168,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="249" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A249">
         <v>6503</v>
       </c>
@@ -28238,7 +28244,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="250" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A250">
         <v>6383</v>
       </c>
@@ -28314,7 +28320,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="251" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A251">
         <v>6383</v>
       </c>
@@ -28390,7 +28396,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="252" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A252">
         <v>6379</v>
       </c>
@@ -28466,7 +28472,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="253" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A253">
         <v>6421</v>
       </c>
@@ -28542,7 +28548,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="254" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A254">
         <v>6372</v>
       </c>
@@ -28618,7 +28624,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="255" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A255">
         <v>6372</v>
       </c>
@@ -28694,7 +28700,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="256" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A256">
         <v>6372</v>
       </c>
@@ -28770,7 +28776,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="257" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A257">
         <v>6439</v>
       </c>
@@ -28846,7 +28852,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="258" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A258">
         <v>6377</v>
       </c>
@@ -28922,7 +28928,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="259" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A259">
         <v>6377</v>
       </c>
@@ -28998,7 +29004,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="260" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A260">
         <v>6377</v>
       </c>
@@ -29074,7 +29080,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="261" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A261">
         <v>6487</v>
       </c>
@@ -29150,7 +29156,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="262" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A262">
         <v>6439</v>
       </c>
@@ -29226,7 +29232,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="263" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A263">
         <v>6371</v>
       </c>
@@ -29302,7 +29308,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="264" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A264">
         <v>6436</v>
       </c>
@@ -29378,7 +29384,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="265" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A265">
         <v>6383</v>
       </c>
@@ -29454,7 +29460,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="266" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A266">
         <v>6383</v>
       </c>
@@ -29530,7 +29536,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="267" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A267">
         <v>6492</v>
       </c>
@@ -29606,7 +29612,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="268" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A268">
         <v>6492</v>
       </c>
@@ -29682,7 +29688,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="269" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A269">
         <v>6487</v>
       </c>
@@ -29758,7 +29764,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="270" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A270">
         <v>6422</v>
       </c>
@@ -29834,7 +29840,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="271" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A271">
         <v>6376</v>
       </c>
@@ -29910,7 +29916,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="272" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A272">
         <v>6452</v>
       </c>
@@ -29986,7 +29992,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="273" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A273">
         <v>6421</v>
       </c>
@@ -30062,7 +30068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="274" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A274">
         <v>6383</v>
       </c>
@@ -30138,7 +30144,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="275" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A275">
         <v>6362</v>
       </c>
@@ -30214,7 +30220,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="276" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A276">
         <v>6540</v>
       </c>
@@ -30290,7 +30296,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="277" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A277">
         <v>6540</v>
       </c>
@@ -30366,7 +30372,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="278" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A278">
         <v>6540</v>
       </c>
@@ -30442,7 +30448,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="279" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A279">
         <v>6488</v>
       </c>
@@ -30518,7 +30524,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="280" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A280">
         <v>6421</v>
       </c>
@@ -30594,7 +30600,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="281" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A281">
         <v>6382</v>
       </c>
@@ -30670,7 +30676,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="282" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A282">
         <v>6382</v>
       </c>
@@ -30746,7 +30752,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="283" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A283">
         <v>6382</v>
       </c>
@@ -30822,7 +30828,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="284" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A284">
         <v>6382</v>
       </c>
@@ -30898,7 +30904,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="285" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A285">
         <v>6362</v>
       </c>
@@ -30974,7 +30980,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="286" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A286">
         <v>6492</v>
       </c>
@@ -31050,7 +31056,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="287" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A287">
         <v>6492</v>
       </c>
@@ -31126,7 +31132,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="288" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A288">
         <v>6492</v>
       </c>
@@ -31202,7 +31208,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="289" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A289">
         <v>6492</v>
       </c>
@@ -31278,7 +31284,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="290" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A290">
         <v>6433</v>
       </c>
@@ -31354,7 +31360,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="291" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A291">
         <v>6381</v>
       </c>
@@ -31430,7 +31436,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="292" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A292">
         <v>6379</v>
       </c>
@@ -31506,7 +31512,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="293" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A293">
         <v>6362</v>
       </c>
@@ -31582,7 +31588,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="294" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A294">
         <v>6376</v>
       </c>
@@ -31658,7 +31664,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="295" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A295">
         <v>6492</v>
       </c>
@@ -31734,7 +31740,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="296" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A296">
         <v>6492</v>
       </c>
@@ -31810,7 +31816,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="297" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A297">
         <v>6421</v>
       </c>
@@ -31886,7 +31892,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="298" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A298">
         <v>6378</v>
       </c>
@@ -31962,7 +31968,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="299" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A299">
         <v>6376</v>
       </c>
@@ -32038,7 +32044,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="300" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A300">
         <v>6376</v>
       </c>
@@ -32114,7 +32120,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="301" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A301">
         <v>6376</v>
       </c>
@@ -32190,7 +32196,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="302" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A302">
         <v>6540</v>
       </c>
@@ -32266,7 +32272,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="303" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A303">
         <v>6540</v>
       </c>
@@ -32342,7 +32348,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="304" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A304">
         <v>6540</v>
       </c>
@@ -32418,7 +32424,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="305" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A305">
         <v>6382</v>
       </c>
@@ -32494,7 +32500,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="306" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A306">
         <v>6382</v>
       </c>
@@ -32570,7 +32576,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="307" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A307">
         <v>6382</v>
       </c>
@@ -32646,7 +32652,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="308" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A308">
         <v>6382</v>
       </c>
@@ -32722,7 +32728,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="309" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A309">
         <v>6379</v>
       </c>
@@ -32798,7 +32804,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="310" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A310">
         <v>6378</v>
       </c>
@@ -32874,7 +32880,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="311" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A311">
         <v>6380</v>
       </c>
@@ -32950,7 +32956,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="312" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="312" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A312">
         <v>6379</v>
       </c>
@@ -33026,7 +33032,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="313" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A313">
         <v>6363</v>
       </c>
@@ -33102,7 +33108,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="314" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="314" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A314">
         <v>6363</v>
       </c>
@@ -33178,7 +33184,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="315" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="315" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A315">
         <v>6623</v>
       </c>
@@ -33254,7 +33260,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="316" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="316" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A316">
         <v>6439</v>
       </c>
@@ -33330,7 +33336,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="317" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="317" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A317">
         <v>6439</v>
       </c>
@@ -33406,7 +33412,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="318" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="318" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A318">
         <v>6439</v>
       </c>
@@ -33482,7 +33488,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="319" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="319" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A319">
         <v>6379</v>
       </c>
@@ -33558,7 +33564,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="320" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="320" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A320">
         <v>6379</v>
       </c>
@@ -33634,7 +33640,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="321" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="321" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A321">
         <v>6517</v>
       </c>
@@ -33710,7 +33716,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="322" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="322" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A322">
         <v>6376</v>
       </c>
@@ -33786,7 +33792,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="323" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="323" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A323">
         <v>6376</v>
       </c>
@@ -33862,7 +33868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="324" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="324" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A324">
         <v>6376</v>
       </c>
@@ -33938,7 +33944,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="325" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="325" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A325">
         <v>6378</v>
       </c>
@@ -34014,7 +34020,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="326" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="326" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A326">
         <v>6378</v>
       </c>
@@ -34090,7 +34096,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="327" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="327" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A327">
         <v>6623</v>
       </c>
@@ -34166,7 +34172,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="328" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="328" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A328">
         <v>6363</v>
       </c>
@@ -34242,7 +34248,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="329" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="329" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A329">
         <v>6363</v>
       </c>
@@ -34318,7 +34324,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="330" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="330" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A330">
         <v>6297</v>
       </c>
@@ -34394,7 +34400,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="331" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="331" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A331">
         <v>6384</v>
       </c>
@@ -34470,7 +34476,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="332" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="332" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A332">
         <v>6492</v>
       </c>
@@ -34546,7 +34552,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="333" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="333" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A333">
         <v>6492</v>
       </c>
@@ -34622,7 +34628,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="334" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="334" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A334">
         <v>6492</v>
       </c>
@@ -34698,7 +34704,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="335" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="335" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A335">
         <v>6492</v>
       </c>
@@ -34774,7 +34780,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="336" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="336" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A336">
         <v>6492</v>
       </c>
@@ -34850,7 +34856,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="337" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="337" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A337">
         <v>6492</v>
       </c>
@@ -34926,7 +34932,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="338" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="338" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A338">
         <v>6381</v>
       </c>
@@ -35002,7 +35008,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="339" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="339" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A339">
         <v>6433</v>
       </c>
@@ -35078,7 +35084,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="340" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="340" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A340">
         <v>6373</v>
       </c>
@@ -35154,7 +35160,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="341" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="341" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A341">
         <v>6378</v>
       </c>
@@ -35230,7 +35236,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="342" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="342" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A342">
         <v>6377</v>
       </c>
@@ -35306,7 +35312,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="343" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="343" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A343">
         <v>6377</v>
       </c>
@@ -35382,7 +35388,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="344" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="344" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A344">
         <v>6377</v>
       </c>
@@ -35458,7 +35464,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="345" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="345" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A345">
         <v>6492</v>
       </c>
@@ -35534,7 +35540,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="346" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="346" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A346">
         <v>6492</v>
       </c>
@@ -35610,7 +35616,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="347" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="347" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A347">
         <v>6376</v>
       </c>
@@ -35686,7 +35692,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="348" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="348" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A348">
         <v>6373</v>
       </c>
@@ -35762,7 +35768,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="349" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="349" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A349">
         <v>6436</v>
       </c>
@@ -35838,7 +35844,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="350" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="350" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A350">
         <v>6421</v>
       </c>
@@ -35914,7 +35920,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="351" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="351" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A351">
         <v>6492</v>
       </c>
@@ -35990,7 +35996,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="352" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="352" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A352">
         <v>6492</v>
       </c>
@@ -36066,7 +36072,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="353" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="353" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A353">
         <v>6377</v>
       </c>
@@ -36142,7 +36148,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="354" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="354" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A354">
         <v>6377</v>
       </c>
@@ -36218,7 +36224,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="355" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="355" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A355">
         <v>6377</v>
       </c>
@@ -36294,7 +36300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="356" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="356" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A356">
         <v>6492</v>
       </c>
@@ -36370,7 +36376,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="357" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="357" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A357">
         <v>6492</v>
       </c>
@@ -36446,7 +36452,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="358" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="358" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A358">
         <v>6433</v>
       </c>
@@ -36522,7 +36528,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="359" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="359" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A359">
         <v>6433</v>
       </c>
@@ -36598,7 +36604,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="360" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="360" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A360">
         <v>6378</v>
       </c>
@@ -36674,7 +36680,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="361" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="361" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A361">
         <v>6378</v>
       </c>
@@ -36750,7 +36756,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="362" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="362" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A362">
         <v>6378</v>
       </c>
@@ -36826,7 +36832,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="363" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="363" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A363">
         <v>6623</v>
       </c>
@@ -36902,7 +36908,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="364" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="364" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A364">
         <v>6484</v>
       </c>
@@ -36978,7 +36984,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="365" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="365" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A365">
         <v>6618</v>
       </c>
@@ -37054,7 +37060,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="366" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="366" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A366">
         <v>6618</v>
       </c>
@@ -37130,7 +37136,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="367" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="367" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A367">
         <v>6492</v>
       </c>
@@ -37206,7 +37212,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="368" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="368" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A368">
         <v>6492</v>
       </c>
@@ -37282,7 +37288,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="369" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="369" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A369">
         <v>6523</v>
       </c>
@@ -37358,7 +37364,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="370" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="370" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A370">
         <v>6523</v>
       </c>
@@ -37434,7 +37440,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="371" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="371" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A371">
         <v>6523</v>
       </c>
@@ -37510,7 +37516,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="372" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="372" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A372">
         <v>6523</v>
       </c>
@@ -37586,7 +37592,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="373" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="373" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A373">
         <v>6492</v>
       </c>
@@ -37662,7 +37668,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="374" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="374" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A374">
         <v>6492</v>
       </c>
@@ -37738,7 +37744,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="375" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="375" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A375">
         <v>6436</v>
       </c>
@@ -37814,7 +37820,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="376" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="376" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A376">
         <v>6538</v>
       </c>
@@ -37890,7 +37896,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="377" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="377" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A377">
         <v>6538</v>
       </c>
@@ -37966,7 +37972,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="378" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="378" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A378">
         <v>6383</v>
       </c>
@@ -38042,7 +38048,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="379" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="379" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A379">
         <v>6377</v>
       </c>
@@ -38118,7 +38124,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="380" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="380" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A380">
         <v>6377</v>
       </c>
@@ -38194,7 +38200,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="381" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="381" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A381">
         <v>6377</v>
       </c>
@@ -38270,7 +38276,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="382" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="382" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A382">
         <v>6493</v>
       </c>
@@ -38346,7 +38352,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="383" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="383" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A383">
         <v>6493</v>
       </c>
@@ -38422,7 +38428,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="384" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="384" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A384">
         <v>6609</v>
       </c>
@@ -38498,7 +38504,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="385" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="385" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A385">
         <v>6492</v>
       </c>
@@ -38574,7 +38580,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="386" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="386" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A386">
         <v>6492</v>
       </c>
@@ -38650,7 +38656,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="387" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="387" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A387">
         <v>6384</v>
       </c>
@@ -38726,7 +38732,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="388" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="388" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A388">
         <v>6376</v>
       </c>
@@ -38802,7 +38808,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="389" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="389" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A389">
         <v>6376</v>
       </c>
@@ -38878,7 +38884,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="390" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="390" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A390">
         <v>6376</v>
       </c>
@@ -38954,7 +38960,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="391" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="391" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A391">
         <v>6492</v>
       </c>
@@ -39030,7 +39036,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="392" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="392" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A392">
         <v>6492</v>
       </c>
@@ -39106,7 +39112,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="393" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="393" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A393">
         <v>6433</v>
       </c>
@@ -39182,7 +39188,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="394" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="394" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A394">
         <v>6436</v>
       </c>
@@ -39258,7 +39264,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="395" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="395" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A395">
         <v>6383</v>
       </c>
@@ -39334,7 +39340,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="396" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="396" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A396">
         <v>6609</v>
       </c>
@@ -39410,7 +39416,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="397" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="397" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A397">
         <v>6381</v>
       </c>
@@ -39486,7 +39492,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="398" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="398" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A398">
         <v>6612</v>
       </c>
@@ -39562,7 +39568,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="399" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="399" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A399">
         <v>6612</v>
       </c>
@@ -39638,7 +39644,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="400" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="400" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A400">
         <v>6433</v>
       </c>
@@ -39714,7 +39720,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="401" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="401" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A401">
         <v>6373</v>
       </c>
@@ -39790,7 +39796,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="402" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="402" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A402">
         <v>6524</v>
       </c>
@@ -39866,7 +39872,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="403" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="403" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A403">
         <v>6503</v>
       </c>
@@ -39942,7 +39948,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="404" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="404" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A404">
         <v>6503</v>
       </c>
@@ -40018,7 +40024,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="405" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="405" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A405">
         <v>6503</v>
       </c>
@@ -40094,7 +40100,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="406" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="406" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A406">
         <v>6485</v>
       </c>
@@ -40170,7 +40176,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="407" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="407" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A407">
         <v>6485</v>
       </c>
@@ -40246,7 +40252,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="408" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="408" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A408">
         <v>6381</v>
       </c>
@@ -40322,7 +40328,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="409" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="409" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A409">
         <v>6618</v>
       </c>
@@ -40398,7 +40404,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="410" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="410" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A410">
         <v>6484</v>
       </c>
@@ -40474,7 +40480,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="411" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="411" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A411">
         <v>6371</v>
       </c>
@@ -40550,7 +40556,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="412" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="412" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A412">
         <v>6612</v>
       </c>
@@ -40626,7 +40632,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="413" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="413" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A413">
         <v>6612</v>
       </c>
@@ -40702,7 +40708,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="414" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="414" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A414">
         <v>6484</v>
       </c>
@@ -40778,7 +40784,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="415" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="415" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A415">
         <v>6618</v>
       </c>
@@ -40854,7 +40860,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="416" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="416" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A416">
         <v>6439</v>
       </c>
@@ -40930,7 +40936,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="417" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="417" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A417">
         <v>6433</v>
       </c>
@@ -41006,7 +41012,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="418" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="418" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A418">
         <v>6439</v>
       </c>
@@ -41082,7 +41088,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="419" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="419" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A419">
         <v>6376</v>
       </c>
@@ -41158,7 +41164,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="420" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="420" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A420">
         <v>6484</v>
       </c>
@@ -41234,7 +41240,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="421" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="421" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A421">
         <v>6609</v>
       </c>
@@ -41310,7 +41316,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="422" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="422" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A422">
         <v>6620</v>
       </c>
@@ -41386,7 +41392,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="423" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="423" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A423">
         <v>6527</v>
       </c>
@@ -41462,7 +41468,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="424" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="424" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A424">
         <v>6433</v>
       </c>
@@ -41538,7 +41544,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="425" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="425" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A425">
         <v>6373</v>
       </c>
@@ -41614,7 +41620,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="426" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="426" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A426">
         <v>6371</v>
       </c>
@@ -41690,7 +41696,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="427" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="427" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A427">
         <v>6484</v>
       </c>
@@ -41766,7 +41772,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="428" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="428" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A428">
         <v>6379</v>
       </c>
@@ -41842,7 +41848,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="429" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="429" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A429">
         <v>6435</v>
       </c>
@@ -41918,7 +41924,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="430" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="430" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A430">
         <v>6373</v>
       </c>
@@ -41994,7 +42000,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="431" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="431" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A431">
         <v>6370</v>
       </c>
@@ -42070,7 +42076,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="432" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="432" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A432">
         <v>6485</v>
       </c>
@@ -42146,7 +42152,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="433" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="433" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A433">
         <v>6485</v>
       </c>
@@ -42222,7 +42228,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="434" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="434" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A434">
         <v>6485</v>
       </c>
@@ -42298,7 +42304,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="435" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="435" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A435">
         <v>6485</v>
       </c>
@@ -42374,7 +42380,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="436" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="436" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A436">
         <v>6439</v>
       </c>
@@ -42450,7 +42456,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="437" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="437" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A437">
         <v>6493</v>
       </c>
@@ -42526,7 +42532,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="438" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="438" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A438">
         <v>6612</v>
       </c>
@@ -42602,7 +42608,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="439" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="439" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A439">
         <v>6452</v>
       </c>
@@ -42678,7 +42684,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="440" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="440" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A440">
         <v>6618</v>
       </c>
@@ -42754,7 +42760,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="441" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="441" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A441">
         <v>6425</v>
       </c>
@@ -42830,7 +42836,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="442" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="442" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A442">
         <v>6486</v>
       </c>
@@ -42906,7 +42912,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="443" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="443" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A443">
         <v>6618</v>
       </c>
@@ -42982,7 +42988,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="444" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="444" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A444">
         <v>6616</v>
       </c>
@@ -43058,7 +43064,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="445" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="445" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A445">
         <v>6534</v>
       </c>
@@ -43134,7 +43140,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="446" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="446" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A446">
         <v>6486</v>
       </c>
@@ -43210,7 +43216,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="447" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="447" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A447">
         <v>6371</v>
       </c>
@@ -43286,7 +43292,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="448" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="448" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A448">
         <v>6381</v>
       </c>
@@ -43362,7 +43368,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="449" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="449" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A449">
         <v>6492</v>
       </c>
@@ -43438,7 +43444,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="450" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="450" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A450">
         <v>6492</v>
       </c>
@@ -43514,7 +43520,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="451" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="451" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A451">
         <v>6529</v>
       </c>
@@ -43590,7 +43596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="452" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="452" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A452">
         <v>6415</v>
       </c>
@@ -43666,7 +43672,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="453" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="453" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A453">
         <v>6492</v>
       </c>
@@ -43742,7 +43748,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="454" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="454" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A454">
         <v>6492</v>
       </c>
@@ -43818,7 +43824,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="455" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="455" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A455">
         <v>6383</v>
       </c>
@@ -43894,7 +43900,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="456" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="456" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A456">
         <v>6415</v>
       </c>
@@ -43970,7 +43976,7 @@
         <v>-200000</v>
       </c>
     </row>
-    <row r="457" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="457" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A457">
         <v>6371</v>
       </c>
@@ -44046,7 +44052,7 @@
         <v>-200000</v>
       </c>
     </row>
-    <row r="458" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="458" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A458">
         <v>6381</v>
       </c>
@@ -44122,7 +44128,7 @@
         <v>-200000</v>
       </c>
     </row>
-    <row r="459" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="459" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A459">
         <v>6425</v>
       </c>
@@ -44198,7 +44204,7 @@
         <v>-200000</v>
       </c>
     </row>
-    <row r="460" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="460" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A460">
         <v>6492</v>
       </c>
@@ -44274,7 +44280,7 @@
         <v>-200000</v>
       </c>
     </row>
-    <row r="461" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="461" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A461">
         <v>6492</v>
       </c>
@@ -44350,7 +44356,7 @@
         <v>-200000</v>
       </c>
     </row>
-    <row r="462" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="462" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A462">
         <v>6492</v>
       </c>
@@ -44426,7 +44432,7 @@
         <v>-200000</v>
       </c>
     </row>
-    <row r="463" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="463" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A463">
         <v>6492</v>
       </c>
@@ -44502,7 +44508,7 @@
         <v>-200000</v>
       </c>
     </row>
-    <row r="464" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="464" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A464">
         <v>6364</v>
       </c>
@@ -44578,7 +44584,7 @@
         <v>-200000</v>
       </c>
     </row>
-    <row r="465" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="465" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A465">
         <v>6491</v>
       </c>
@@ -44654,7 +44660,7 @@
         <v>-200000</v>
       </c>
     </row>
-    <row r="466" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="466" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A466">
         <v>6379</v>
       </c>
@@ -44730,7 +44736,7 @@
         <v>-200000</v>
       </c>
     </row>
-    <row r="467" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="467" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A467">
         <v>6543</v>
       </c>
@@ -44806,7 +44812,7 @@
         <v>-200000</v>
       </c>
     </row>
-    <row r="468" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="468" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A468">
         <v>6485</v>
       </c>
@@ -44882,7 +44888,7 @@
         <v>-200000</v>
       </c>
     </row>
-    <row r="469" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="469" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A469">
         <v>6485</v>
       </c>
@@ -44958,7 +44964,7 @@
         <v>-200000</v>
       </c>
     </row>
-    <row r="470" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="470" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A470">
         <v>6620</v>
       </c>
@@ -45034,7 +45040,7 @@
         <v>-200000</v>
       </c>
     </row>
-    <row r="471" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="471" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A471">
         <v>6383</v>
       </c>
@@ -45110,7 +45116,7 @@
         <v>-200000</v>
       </c>
     </row>
-    <row r="472" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="472" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A472">
         <v>6496</v>
       </c>
@@ -45186,7 +45192,7 @@
         <v>-400000</v>
       </c>
     </row>
-    <row r="473" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="473" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A473">
         <v>6496</v>
       </c>
@@ -45262,7 +45268,7 @@
         <v>-400000</v>
       </c>
     </row>
-    <row r="474" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="474" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A474">
         <v>6496</v>
       </c>
@@ -45338,7 +45344,7 @@
         <v>-400000</v>
       </c>
     </row>
-    <row r="475" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="475" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A475">
         <v>6621</v>
       </c>
@@ -45414,7 +45420,7 @@
         <v>-400000</v>
       </c>
     </row>
-    <row r="476" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="476" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A476">
         <v>6485</v>
       </c>
@@ -45490,7 +45496,7 @@
         <v>-400000</v>
       </c>
     </row>
-    <row r="477" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="477" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A477">
         <v>6485</v>
       </c>
@@ -45566,7 +45572,7 @@
         <v>-400000</v>
       </c>
     </row>
-    <row r="478" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="478" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A478">
         <v>6618</v>
       </c>
@@ -45642,7 +45648,7 @@
         <v>-400000</v>
       </c>
     </row>
-    <row r="479" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="479" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A479">
         <v>6616</v>
       </c>
@@ -45718,7 +45724,7 @@
         <v>-600000</v>
       </c>
     </row>
-    <row r="480" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="480" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A480">
         <v>6415</v>
       </c>
@@ -45794,7 +45800,7 @@
         <v>-600000</v>
       </c>
     </row>
-    <row r="481" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="481" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A481">
         <v>6618</v>
       </c>
@@ -45870,7 +45876,7 @@
         <v>-600000</v>
       </c>
     </row>
-    <row r="482" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="482" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A482">
         <v>6297</v>
       </c>
@@ -45946,7 +45952,7 @@
         <v>-800000</v>
       </c>
     </row>
-    <row r="483" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="483" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A483">
         <v>6415</v>
       </c>
@@ -46022,7 +46028,7 @@
         <v>-1000000</v>
       </c>
     </row>
-    <row r="484" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="484" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A484">
         <v>6496</v>
       </c>
@@ -46098,7 +46104,7 @@
         <v>-1200000</v>
       </c>
     </row>
-    <row r="485" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="485" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A485">
         <v>6487</v>
       </c>
@@ -46174,7 +46180,7 @@
         <v>-1400000</v>
       </c>
     </row>
-    <row r="486" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="486" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A486">
         <v>6492</v>
       </c>
@@ -46250,7 +46256,7 @@
         <v>-1400000</v>
       </c>
     </row>
-    <row r="487" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="487" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A487">
         <v>6492</v>
       </c>
@@ -46326,7 +46332,7 @@
         <v>-1400000</v>
       </c>
     </row>
-    <row r="488" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="488" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A488">
         <v>6543</v>
       </c>
@@ -46402,7 +46408,7 @@
         <v>-1600000</v>
       </c>
     </row>
-    <row r="489" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="489" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A489">
         <v>6485</v>
       </c>
@@ -46478,7 +46484,7 @@
         <v>-1800000</v>
       </c>
     </row>
-    <row r="490" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="490" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A490">
         <v>6485</v>
       </c>
@@ -46554,7 +46560,7 @@
         <v>-1800000</v>
       </c>
     </row>
-    <row r="491" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="491" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A491">
         <v>6430</v>
       </c>
@@ -46630,7 +46636,7 @@
         <v>-2600000</v>
       </c>
     </row>
-    <row r="492" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="492" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A492">
         <v>6430</v>
       </c>
@@ -46706,7 +46712,7 @@
         <v>-2600000</v>
       </c>
     </row>
-    <row r="493" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="493" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A493">
         <v>6430</v>
       </c>
@@ -46782,7 +46788,7 @@
         <v>-2600000</v>
       </c>
     </row>
-    <row r="494" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="494" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A494">
         <v>6297</v>
       </c>
@@ -46858,7 +46864,7 @@
         <v>-8200000</v>
       </c>
     </row>
-    <row r="495" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="495" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A495">
         <v>6430</v>
       </c>
@@ -46934,7 +46940,7 @@
         <v>-8400000</v>
       </c>
     </row>
-    <row r="496" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="496" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A496">
         <v>6324</v>
       </c>
@@ -47013,7 +47019,7 @@
     <row r="497" spans="22:22" x14ac:dyDescent="0.3">
       <c r="V497" s="1">
         <f>SUBTOTAL(109,Tabla1[Diferencia])</f>
-        <v>-45026469.900000006</v>
+        <v>317500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>